<commit_message>
Sayan Saha Manual Testing final Deliverables
</commit_message>
<xml_diff>
--- a/Day 2_Manual Testing/Sayan_Saha_Magicbricks_Group4.xlsx
+++ b/Day 2_Manual Testing/Sayan_Saha_Magicbricks_Group4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sayan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FDB588-E71F-4FC7-85DD-853F4C71E501}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF04AD86-B9E4-44FE-BBDF-97351F52B79C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="357">
   <si>
     <t>Issue Type</t>
   </si>
@@ -576,18 +576,6 @@
     <t>Project cards must show all required fields and a valid enquiry must be submitted successfully</t>
   </si>
   <si>
-    <t>1. Hover 'Buy' &gt; click 'New Projects'
-2. Inspect 3 project listing cards
-3. Open a project &gt; click 'Enquire Now'
-4. Fill Name='Test User', Mobile=9876543210, Message='Interested'
-5. Click Submit</t>
-  </si>
-  <si>
-    <t>Name: Test User
-Mobile: 9876543210
-Message: Interested in 3 BHK</t>
-  </si>
-  <si>
     <t>Each card shows project name, builder name, RERA number, launch date, and starting price. Enquiry submitted. Confirmation message displayed. Lead visible in My Enquiries.</t>
   </si>
   <si>
@@ -713,17 +701,6 @@
   </si>
   <si>
     <t>BHK filter must be absent, commercial filters present, and valid enquiry must submit successfully</t>
-  </si>
-  <si>
-    <t>1. Hover 'Buy' &gt; click 'Office Space in Mumbai'
-2. Check filter panel for BHK filter
-3. Inspect 5 cards
-4. Open a listing &gt; submit enquiry with Name='Amit', Mobile=9876543210, Message='Interested'</t>
-  </si>
-  <si>
-    <t>Name: Amit
-Mobile: 9876543210
-Message: Interested in office space</t>
   </si>
   <si>
     <t>BHK filter absent. Commercial filters visible (carpet area, furnishing, floor). All 5 cards are Office Space type. Enquiry submitted with confirmation shown.</t>
@@ -1422,6 +1399,35 @@
 4. Click 'Continue to Post'
 Expected Result:
 Form submission is blocked. Validation error 'Please select the no. of bedrooms' appears adjacent to the Bedrooms field. Field is highlighted in error state. No listing is created.</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>1. Hover 'Buy' &gt; click 'New Projects'
+2. Inspect 3 project listing cards
+3. Open a project &gt; click 'Enquire Now'
+4. Fill Name='Test User', Mobile=9876543210, Email = "testuser@gmail.com"
+5. Click Submit</t>
+  </si>
+  <si>
+    <t>Name: Test User
+Mobile: 9876543210
+Email: "testuser@gmail.com"</t>
+  </si>
+  <si>
+    <t>1. Hover 'Buy' &gt; click 'Office Space in Mumbai'
+2. Check filter panel for BHK filter
+3. Inspect 5 cards
+4. Open a listing &gt; submit enquiry with Name='Amit', Mobile=9876543210, Email="amit@gmail.com"</t>
+  </si>
+  <si>
+    <t>Name: Amit
+Mobile: 9876543210
+Email: "amit@gmail.com"</t>
+  </si>
+  <si>
+    <t>Test Case Passed Successfully</t>
   </si>
 </sst>
 </file>
@@ -1727,7 +1733,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1856,22 +1862,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1879,29 +1891,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -2226,7 +2216,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>4</v>
@@ -2237,7 +2227,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>4</v>
@@ -2248,7 +2238,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>4</v>
@@ -2259,7 +2249,7 @@
         <v>110</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>11</v>
@@ -2270,7 +2260,7 @@
         <v>111</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>11</v>
@@ -2292,7 +2282,7 @@
         <v>113</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>4</v>
@@ -2303,7 +2293,7 @@
         <v>114</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>4</v>
@@ -2314,7 +2304,7 @@
         <v>115</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>4</v>
@@ -2325,7 +2315,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>4</v>
@@ -2336,7 +2326,7 @@
         <v>117</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>4</v>
@@ -2347,7 +2337,7 @@
         <v>118</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>4</v>
@@ -2421,10 +2411,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="33" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B22" s="34" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C22" s="33" t="s">
         <v>4</v>
@@ -2432,10 +2422,10 @@
     </row>
     <row r="23" spans="1:3" ht="27.6">
       <c r="A23" s="35" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="B23" s="36" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="C23" s="35" t="s">
         <v>4</v>
@@ -2443,10 +2433,10 @@
     </row>
     <row r="24" spans="1:3" ht="43.2">
       <c r="A24" s="37" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C24" s="38" t="s">
         <v>4</v>
@@ -2454,10 +2444,10 @@
     </row>
     <row r="25" spans="1:3" ht="43.2">
       <c r="A25" s="37" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>4</v>
@@ -2465,10 +2455,10 @@
     </row>
     <row r="26" spans="1:3" ht="43.2">
       <c r="A26" s="37" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="C26" s="38" t="s">
         <v>11</v>
@@ -2495,7 +2485,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="82.8" customHeight="1">
       <c r="A1" s="20" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>12</v>
@@ -2507,7 +2497,7 @@
         <v>14</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F1" s="20" t="s">
         <v>15</v>
@@ -2515,7 +2505,7 @@
     </row>
     <row r="2" spans="1:6" ht="151.80000000000001" customHeight="1">
       <c r="A2" s="39" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B2" s="39" t="s">
         <v>50</v>
@@ -2524,18 +2514,18 @@
         <v>51</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E2" s="18">
         <v>1</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="256.2" customHeight="1">
       <c r="A3" s="39" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B3" s="39" t="s">
         <v>54</v>
@@ -2544,18 +2534,18 @@
         <v>55</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E3" s="18">
         <v>2</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="117" customHeight="1">
       <c r="A4" s="39" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B4" s="39" t="s">
         <v>58</v>
@@ -2564,18 +2554,18 @@
         <v>59</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E4" s="18">
         <v>2</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>350</v>
+        <v>346</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="54.6" customHeight="1">
       <c r="A5" s="39" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B5" s="39" t="s">
         <v>62</v>
@@ -2584,18 +2574,18 @@
         <v>63</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E5" s="18">
         <v>1</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="79.2" customHeight="1">
       <c r="A6" s="39" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B6" s="39" t="s">
         <v>66</v>
@@ -2604,18 +2594,18 @@
         <v>67</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E6" s="18">
         <v>2</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>351</v>
+        <v>347</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="87" customHeight="1">
       <c r="A7" s="39" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B7" s="39" t="s">
         <v>70</v>
@@ -2624,18 +2614,18 @@
         <v>71</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E7" s="18">
         <v>1</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="67.8" customHeight="1">
       <c r="A8" s="39" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="B8" s="39" t="s">
         <v>74</v>
@@ -2644,18 +2634,18 @@
         <v>75</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E8" s="18">
         <v>1</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="84" customHeight="1">
       <c r="A9" s="39" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B9" s="39" t="s">
         <v>78</v>
@@ -2664,18 +2654,18 @@
         <v>79</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E9" s="18">
         <v>1</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="82.2" customHeight="1">
       <c r="A10" s="39" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B10" s="39" t="s">
         <v>83</v>
@@ -2684,18 +2674,18 @@
         <v>84</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E10" s="18">
         <v>2</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="85.2" customHeight="1">
       <c r="A11" s="39" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B11" s="39" t="s">
         <v>87</v>
@@ -2704,18 +2694,18 @@
         <v>88</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E11" s="18">
         <v>2</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>353</v>
+        <v>349</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="88.2" customHeight="1">
       <c r="A12" s="39" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B12" s="39" t="s">
         <v>92</v>
@@ -2724,18 +2714,18 @@
         <v>93</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E12" s="18">
         <v>1</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="99.6" customHeight="1">
       <c r="A13" s="39" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B13" s="39" t="s">
         <v>96</v>
@@ -2744,18 +2734,18 @@
         <v>97</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E13" s="18">
         <v>1</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="94.2" customHeight="1">
       <c r="A14" s="39" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B14" s="39" t="s">
         <v>100</v>
@@ -2764,18 +2754,18 @@
         <v>101</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E14" s="18">
         <v>1</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="61.8" customHeight="1">
       <c r="A15" s="39" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B15" s="39" t="s">
         <v>102</v>
@@ -2784,18 +2774,18 @@
         <v>103</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E15" s="18">
         <v>1</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="95.4" hidden="1" customHeight="1">
       <c r="A16" s="39" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B16" s="39" t="s">
         <v>104</v>
@@ -2804,18 +2794,18 @@
         <v>105</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E16" s="18">
         <v>2</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="91.8" customHeight="1">
       <c r="A17" s="39" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B17" s="39" t="s">
         <v>106</v>
@@ -2824,33 +2814,33 @@
         <v>107</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E17" s="18">
         <v>1</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="72" customHeight="1">
       <c r="A18" s="39" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E18" s="18">
         <v>3</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>354</v>
+        <v>350</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="94.8" customHeight="1"/>
@@ -2901,6 +2891,7 @@
     <col min="5" max="5" width="20.109375" customWidth="1"/>
     <col min="6" max="6" width="17" customWidth="1"/>
     <col min="7" max="7" width="18.5546875" customWidth="1"/>
+    <col min="12" max="12" width="20.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="84">
@@ -2946,7 +2937,7 @@
     </row>
     <row r="2" spans="1:13" ht="72">
       <c r="A2" s="22" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -2983,18 +2974,22 @@
       <c r="G3" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="H3" s="25"/>
+      <c r="H3" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I3" s="24"/>
       <c r="J3" s="25"/>
       <c r="K3" s="24"/>
-      <c r="L3" s="25"/>
+      <c r="L3" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M3" s="24" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="72">
       <c r="A4" s="22" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -3031,11 +3026,15 @@
       <c r="G5" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="H5" s="27"/>
+      <c r="H5" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I5" s="28"/>
       <c r="J5" s="27"/>
       <c r="K5" s="28"/>
-      <c r="L5" s="27"/>
+      <c r="L5" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M5" s="28" t="s">
         <v>54</v>
       </c>
@@ -3062,18 +3061,22 @@
       <c r="G6" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="H6" s="30"/>
+      <c r="H6" s="52" t="s">
+        <v>351</v>
+      </c>
       <c r="I6" s="29"/>
       <c r="J6" s="30"/>
       <c r="K6" s="29"/>
-      <c r="L6" s="30"/>
+      <c r="L6" s="29" t="s">
+        <v>356</v>
+      </c>
       <c r="M6" s="29" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="72">
       <c r="A7" s="22" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
@@ -3110,11 +3113,15 @@
       <c r="G8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="H8" s="27"/>
+      <c r="H8" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I8" s="28"/>
       <c r="J8" s="27"/>
       <c r="K8" s="28"/>
-      <c r="L8" s="27"/>
+      <c r="L8" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M8" s="28" t="s">
         <v>58</v>
       </c>
@@ -3141,18 +3148,22 @@
       <c r="G9" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="30"/>
+      <c r="H9" s="52" t="s">
+        <v>351</v>
+      </c>
       <c r="I9" s="29"/>
       <c r="J9" s="30"/>
       <c r="K9" s="29"/>
-      <c r="L9" s="30"/>
+      <c r="L9" s="29" t="s">
+        <v>356</v>
+      </c>
       <c r="M9" s="29" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="84">
       <c r="A10" s="22" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
@@ -3189,18 +3200,22 @@
       <c r="G11" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="H11" s="27"/>
+      <c r="H11" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I11" s="28"/>
       <c r="J11" s="27"/>
       <c r="K11" s="28"/>
-      <c r="L11" s="27"/>
+      <c r="L11" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M11" s="28" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="84">
       <c r="A12" s="22" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
@@ -3215,7 +3230,7 @@
       <c r="L12" s="26"/>
       <c r="M12" s="26"/>
     </row>
-    <row r="13" spans="1:13" ht="145.19999999999999">
+    <row r="13" spans="1:13" ht="158.4">
       <c r="A13" s="24" t="s">
         <v>61</v>
       </c>
@@ -3229,19 +3244,23 @@
         <v>168</v>
       </c>
       <c r="E13" s="25" t="s">
+        <v>352</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>353</v>
+      </c>
+      <c r="G13" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="F13" s="25" t="s">
-        <v>170</v>
-      </c>
-      <c r="G13" s="25" t="s">
-        <v>171</v>
-      </c>
-      <c r="H13" s="25"/>
+      <c r="H13" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I13" s="24"/>
       <c r="J13" s="25"/>
       <c r="K13" s="24"/>
-      <c r="L13" s="25"/>
+      <c r="L13" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M13" s="24" t="s">
         <v>66</v>
       </c>
@@ -3257,29 +3276,33 @@
         <v>167</v>
       </c>
       <c r="D14" s="31" t="s">
+        <v>170</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>171</v>
+      </c>
+      <c r="F14" s="31" t="s">
         <v>172</v>
       </c>
-      <c r="E14" s="31" t="s">
+      <c r="G14" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="F14" s="31" t="s">
-        <v>174</v>
-      </c>
-      <c r="G14" s="31" t="s">
-        <v>175</v>
-      </c>
-      <c r="H14" s="31"/>
+      <c r="H14" s="52" t="s">
+        <v>351</v>
+      </c>
       <c r="I14" s="32"/>
       <c r="J14" s="31"/>
       <c r="K14" s="32"/>
-      <c r="L14" s="31"/>
+      <c r="L14" s="29" t="s">
+        <v>356</v>
+      </c>
       <c r="M14" s="32" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="84">
       <c r="A15" s="22" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -3299,35 +3322,39 @@
         <v>65</v>
       </c>
       <c r="B16" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>175</v>
+      </c>
+      <c r="D16" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="E16" s="25" t="s">
         <v>177</v>
       </c>
-      <c r="D16" s="25" t="s">
+      <c r="F16" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="E16" s="25" t="s">
+      <c r="G16" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="F16" s="25" t="s">
-        <v>180</v>
-      </c>
-      <c r="G16" s="25" t="s">
-        <v>181</v>
-      </c>
-      <c r="H16" s="25"/>
+      <c r="H16" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I16" s="24"/>
       <c r="J16" s="25"/>
       <c r="K16" s="24"/>
-      <c r="L16" s="25"/>
+      <c r="L16" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M16" s="24" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="84">
       <c r="A17" s="22" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
@@ -3347,35 +3374,39 @@
         <v>68</v>
       </c>
       <c r="B18" s="25" t="s">
+        <v>180</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>181</v>
+      </c>
+      <c r="D18" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="E18" s="25" t="s">
         <v>183</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="F18" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="E18" s="25" t="s">
+      <c r="G18" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="F18" s="25" t="s">
-        <v>186</v>
-      </c>
-      <c r="G18" s="25" t="s">
-        <v>187</v>
-      </c>
-      <c r="H18" s="25"/>
+      <c r="H18" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I18" s="24"/>
       <c r="J18" s="25"/>
       <c r="K18" s="24"/>
-      <c r="L18" s="25"/>
+      <c r="L18" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M18" s="24" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="60">
       <c r="A19" s="22" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -3395,35 +3426,39 @@
         <v>69</v>
       </c>
       <c r="B20" s="27" t="s">
+        <v>186</v>
+      </c>
+      <c r="C20" s="27" t="s">
+        <v>187</v>
+      </c>
+      <c r="D20" s="27" t="s">
         <v>188</v>
-      </c>
-      <c r="C20" s="27" t="s">
-        <v>189</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>190</v>
       </c>
       <c r="E20" s="27" t="s">
         <v>80</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G20" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="H20" s="27"/>
+        <v>190</v>
+      </c>
+      <c r="H20" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I20" s="28"/>
       <c r="J20" s="27"/>
       <c r="K20" s="28"/>
-      <c r="L20" s="27"/>
+      <c r="L20" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M20" s="28" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="84">
       <c r="A21" s="22" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -3443,28 +3478,32 @@
         <v>72</v>
       </c>
       <c r="B22" s="25" t="s">
+        <v>191</v>
+      </c>
+      <c r="C22" s="25" t="s">
+        <v>192</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>193</v>
       </c>
-      <c r="C22" s="25" t="s">
+      <c r="E22" s="25" t="s">
         <v>194</v>
       </c>
-      <c r="D22" s="25" t="s">
+      <c r="F22" s="25" t="s">
         <v>195</v>
       </c>
-      <c r="E22" s="25" t="s">
+      <c r="G22" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="F22" s="25" t="s">
-        <v>197</v>
-      </c>
-      <c r="G22" s="25" t="s">
-        <v>198</v>
-      </c>
-      <c r="H22" s="25"/>
+      <c r="H22" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I22" s="24"/>
       <c r="J22" s="25"/>
       <c r="K22" s="24"/>
-      <c r="L22" s="25"/>
+      <c r="L22" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M22" s="24" t="s">
         <v>83</v>
       </c>
@@ -3474,35 +3513,39 @@
         <v>73</v>
       </c>
       <c r="B23" s="31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C23" s="31" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D23" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="E23" s="31" t="s">
+        <v>198</v>
+      </c>
+      <c r="F23" s="31" t="s">
+        <v>284</v>
+      </c>
+      <c r="G23" s="31" t="s">
         <v>199</v>
       </c>
-      <c r="E23" s="31" t="s">
-        <v>200</v>
-      </c>
-      <c r="F23" s="31" t="s">
-        <v>288</v>
-      </c>
-      <c r="G23" s="31" t="s">
-        <v>201</v>
-      </c>
-      <c r="H23" s="31"/>
+      <c r="H23" s="52" t="s">
+        <v>351</v>
+      </c>
       <c r="I23" s="32"/>
       <c r="J23" s="31"/>
       <c r="K23" s="32"/>
-      <c r="L23" s="31"/>
+      <c r="L23" s="29" t="s">
+        <v>356</v>
+      </c>
       <c r="M23" s="32" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:13" ht="84">
       <c r="A24" s="22" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -3517,33 +3560,37 @@
       <c r="L24" s="26"/>
       <c r="M24" s="26"/>
     </row>
-    <row r="25" spans="1:13" ht="145.19999999999999">
+    <row r="25" spans="1:13" ht="158.4">
       <c r="A25" s="24" t="s">
         <v>76</v>
       </c>
       <c r="B25" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="C25" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="C25" s="25" t="s">
+      <c r="E25" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="F25" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="G25" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="D25" s="25" t="s">
-        <v>204</v>
-      </c>
-      <c r="E25" s="25" t="s">
-        <v>205</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>206</v>
-      </c>
-      <c r="G25" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="H25" s="25"/>
+      <c r="H25" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I25" s="24"/>
       <c r="J25" s="25"/>
       <c r="K25" s="24"/>
-      <c r="L25" s="25"/>
+      <c r="L25" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M25" s="24" t="s">
         <v>87</v>
       </c>
@@ -3553,35 +3600,39 @@
         <v>77</v>
       </c>
       <c r="B26" s="31" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E26" s="31" t="s">
         <v>90</v>
       </c>
       <c r="F26" s="31" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="G26" s="31" t="s">
-        <v>210</v>
-      </c>
-      <c r="H26" s="31"/>
+        <v>206</v>
+      </c>
+      <c r="H26" s="52" t="s">
+        <v>351</v>
+      </c>
       <c r="I26" s="32"/>
       <c r="J26" s="31"/>
       <c r="K26" s="32"/>
-      <c r="L26" s="31"/>
+      <c r="L26" s="29" t="s">
+        <v>356</v>
+      </c>
       <c r="M26" s="32" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="84">
       <c r="A27" s="22" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -3601,35 +3652,39 @@
         <v>81</v>
       </c>
       <c r="B28" s="25" t="s">
+        <v>207</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>208</v>
+      </c>
+      <c r="D28" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="E28" s="25" t="s">
+        <v>210</v>
+      </c>
+      <c r="F28" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="C28" s="25" t="s">
+      <c r="G28" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="D28" s="25" t="s">
-        <v>213</v>
-      </c>
-      <c r="E28" s="25" t="s">
-        <v>214</v>
-      </c>
-      <c r="F28" s="25" t="s">
-        <v>215</v>
-      </c>
-      <c r="G28" s="25" t="s">
-        <v>216</v>
-      </c>
-      <c r="H28" s="25"/>
+      <c r="H28" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I28" s="24"/>
       <c r="J28" s="25"/>
       <c r="K28" s="24"/>
-      <c r="L28" s="25"/>
+      <c r="L28" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M28" s="24" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:13" ht="72">
       <c r="A29" s="22" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="B29" s="23"/>
       <c r="C29" s="23"/>
@@ -3649,35 +3704,39 @@
         <v>82</v>
       </c>
       <c r="B30" s="25" t="s">
+        <v>213</v>
+      </c>
+      <c r="C30" s="25" t="s">
+        <v>214</v>
+      </c>
+      <c r="D30" s="25" t="s">
+        <v>215</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>216</v>
+      </c>
+      <c r="F30" s="25" t="s">
         <v>217</v>
       </c>
-      <c r="C30" s="25" t="s">
+      <c r="G30" s="25" t="s">
         <v>218</v>
       </c>
-      <c r="D30" s="25" t="s">
-        <v>219</v>
-      </c>
-      <c r="E30" s="25" t="s">
-        <v>220</v>
-      </c>
-      <c r="F30" s="25" t="s">
-        <v>221</v>
-      </c>
-      <c r="G30" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="H30" s="25"/>
+      <c r="H30" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I30" s="24"/>
       <c r="J30" s="25"/>
       <c r="K30" s="24"/>
-      <c r="L30" s="25"/>
+      <c r="L30" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M30" s="24" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="31" spans="1:13" ht="72">
       <c r="A31" s="22" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="B31" s="26"/>
       <c r="C31" s="26"/>
@@ -3700,32 +3759,36 @@
         <v>101</v>
       </c>
       <c r="C32" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="D32" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E32" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="G32" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="D32" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="E32" s="27" t="s">
-        <v>225</v>
-      </c>
-      <c r="F32" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="G32" s="27" t="s">
-        <v>227</v>
-      </c>
-      <c r="H32" s="27"/>
+      <c r="H32" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="27"/>
       <c r="K32" s="28"/>
-      <c r="L32" s="27"/>
+      <c r="L32" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M32" s="28" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="84">
       <c r="A33" s="22" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B33" s="26"/>
       <c r="C33" s="26"/>
@@ -3745,35 +3808,39 @@
         <v>86</v>
       </c>
       <c r="B34" s="25" t="s">
+        <v>224</v>
+      </c>
+      <c r="C34" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="D34" s="25" t="s">
+        <v>226</v>
+      </c>
+      <c r="E34" s="25" t="s">
+        <v>227</v>
+      </c>
+      <c r="F34" s="25" t="s">
         <v>228</v>
       </c>
-      <c r="C34" s="25" t="s">
+      <c r="G34" s="25" t="s">
         <v>229</v>
       </c>
-      <c r="D34" s="25" t="s">
-        <v>230</v>
-      </c>
-      <c r="E34" s="25" t="s">
-        <v>231</v>
-      </c>
-      <c r="F34" s="25" t="s">
-        <v>232</v>
-      </c>
-      <c r="G34" s="25" t="s">
-        <v>233</v>
-      </c>
-      <c r="H34" s="25"/>
+      <c r="H34" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I34" s="24"/>
       <c r="J34" s="25"/>
       <c r="K34" s="24"/>
-      <c r="L34" s="25"/>
+      <c r="L34" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M34" s="24" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:13" ht="72">
       <c r="A35" s="22" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="B35" s="23"/>
       <c r="C35" s="23"/>
@@ -3796,25 +3863,29 @@
         <v>105</v>
       </c>
       <c r="C36" s="25" t="s">
+        <v>230</v>
+      </c>
+      <c r="D36" s="25" t="s">
+        <v>231</v>
+      </c>
+      <c r="E36" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="F36" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="G36" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="D36" s="25" t="s">
-        <v>235</v>
-      </c>
-      <c r="E36" s="25" t="s">
-        <v>236</v>
-      </c>
-      <c r="F36" s="25" t="s">
-        <v>237</v>
-      </c>
-      <c r="G36" s="25" t="s">
-        <v>238</v>
-      </c>
-      <c r="H36" s="25"/>
+      <c r="H36" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I36" s="24"/>
       <c r="J36" s="25"/>
       <c r="K36" s="24"/>
-      <c r="L36" s="25"/>
+      <c r="L36" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M36" s="24" t="s">
         <v>104</v>
       </c>
@@ -3827,32 +3898,36 @@
         <v>105</v>
       </c>
       <c r="C37" s="25" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D37" s="25" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="F37" s="25" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="G37" s="25" t="s">
-        <v>242</v>
-      </c>
-      <c r="H37" s="25"/>
+        <v>238</v>
+      </c>
+      <c r="H37" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I37" s="24"/>
       <c r="J37" s="25"/>
       <c r="K37" s="24"/>
-      <c r="L37" s="25"/>
+      <c r="L37" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M37" s="24" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="38" spans="1:13" ht="84">
       <c r="A38" s="22" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="B38" s="23"/>
       <c r="C38" s="23"/>
@@ -3872,35 +3947,39 @@
         <v>94</v>
       </c>
       <c r="B39" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>240</v>
+      </c>
+      <c r="D39" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>242</v>
+      </c>
+      <c r="F39" s="25" t="s">
         <v>243</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="G39" s="25" t="s">
         <v>244</v>
       </c>
-      <c r="D39" s="25" t="s">
-        <v>245</v>
-      </c>
-      <c r="E39" s="25" t="s">
-        <v>246</v>
-      </c>
-      <c r="F39" s="25" t="s">
-        <v>247</v>
-      </c>
-      <c r="G39" s="25" t="s">
-        <v>248</v>
-      </c>
-      <c r="H39" s="25"/>
+      <c r="H39" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I39" s="24"/>
       <c r="J39" s="25"/>
       <c r="K39" s="24"/>
-      <c r="L39" s="25"/>
+      <c r="L39" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M39" s="24" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="40" spans="1:13" ht="60">
       <c r="A40" s="40" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="B40" s="23"/>
       <c r="C40" s="23"/>
@@ -3920,30 +3999,34 @@
         <v>95</v>
       </c>
       <c r="B41" s="27" t="s">
+        <v>321</v>
+      </c>
+      <c r="C41" s="27" t="s">
+        <v>322</v>
+      </c>
+      <c r="D41" s="27" t="s">
+        <v>323</v>
+      </c>
+      <c r="E41" s="27" t="s">
+        <v>324</v>
+      </c>
+      <c r="F41" s="27" t="s">
         <v>325</v>
       </c>
-      <c r="C41" s="27" t="s">
+      <c r="G41" s="27" t="s">
         <v>326</v>
       </c>
-      <c r="D41" s="27" t="s">
-        <v>327</v>
-      </c>
-      <c r="E41" s="27" t="s">
-        <v>328</v>
-      </c>
-      <c r="F41" s="27" t="s">
-        <v>329</v>
-      </c>
-      <c r="G41" s="27" t="s">
-        <v>330</v>
-      </c>
-      <c r="H41" s="27"/>
+      <c r="H41" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I41" s="27"/>
       <c r="J41" s="27"/>
       <c r="K41" s="27"/>
-      <c r="L41" s="27"/>
+      <c r="L41" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M41" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="198">
@@ -3951,30 +4034,34 @@
         <v>98</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C42" s="27" t="s">
+        <v>327</v>
+      </c>
+      <c r="D42" s="27" t="s">
+        <v>328</v>
+      </c>
+      <c r="E42" s="27" t="s">
+        <v>329</v>
+      </c>
+      <c r="F42" s="27" t="s">
+        <v>330</v>
+      </c>
+      <c r="G42" s="27" t="s">
         <v>331</v>
       </c>
-      <c r="D42" s="27" t="s">
-        <v>332</v>
-      </c>
-      <c r="E42" s="27" t="s">
-        <v>333</v>
-      </c>
-      <c r="F42" s="27" t="s">
-        <v>334</v>
-      </c>
-      <c r="G42" s="27" t="s">
-        <v>335</v>
-      </c>
-      <c r="H42" s="27"/>
+      <c r="H42" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I42" s="27"/>
       <c r="J42" s="27"/>
       <c r="K42" s="27"/>
-      <c r="L42" s="27"/>
+      <c r="L42" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M42" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="184.8">
@@ -3982,34 +4069,39 @@
         <v>99</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="D43" s="27" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="E43" s="27" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="F43" s="27" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="G43" s="27" t="s">
-        <v>339</v>
-      </c>
-      <c r="H43" s="27"/>
+        <v>335</v>
+      </c>
+      <c r="H43" s="51" t="s">
+        <v>351</v>
+      </c>
       <c r="I43" s="27"/>
       <c r="J43" s="27"/>
       <c r="K43" s="27"/>
-      <c r="L43" s="27"/>
+      <c r="L43" s="24" t="s">
+        <v>356</v>
+      </c>
       <c r="M43" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4048,22 +4140,22 @@
     </row>
     <row r="2" spans="1:6" ht="69.900000000000006" customHeight="1">
       <c r="A2" s="42" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="F2" s="42" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4115,13 +4207,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="42" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B2" s="42" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="D2" s="42" t="s">
         <v>49</v>
@@ -4139,7 +4231,7 @@
         <v>54</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D3" s="42" t="s">
         <v>52</v>
@@ -4171,7 +4263,7 @@
         <v>58</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>56</v>
@@ -4203,7 +4295,7 @@
         <v>62</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="D7" s="42" t="s">
         <v>60</v>
@@ -4221,7 +4313,7 @@
         <v>66</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="D8" s="42" t="s">
         <v>61</v>
@@ -4249,13 +4341,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="42" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="B10" s="42" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="D10" s="42" t="s">
         <v>65</v>
@@ -4273,7 +4365,7 @@
         <v>74</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="D11" s="42" t="s">
         <v>68</v>
@@ -4291,7 +4383,7 @@
         <v>78</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="D12" s="42" t="s">
         <v>69</v>
@@ -4309,7 +4401,7 @@
         <v>83</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>72</v>
@@ -4341,7 +4433,7 @@
         <v>87</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>76</v>
@@ -4373,7 +4465,7 @@
         <v>92</v>
       </c>
       <c r="C17" s="42" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="D17" s="42" t="s">
         <v>81</v>
@@ -4387,13 +4479,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="42" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="B18" s="42" t="s">
         <v>96</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="D18" s="42" t="s">
         <v>82</v>
@@ -4411,7 +4503,7 @@
         <v>100</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="D19" s="42" t="s">
         <v>85</v>
@@ -4429,7 +4521,7 @@
         <v>102</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="D20" s="42" t="s">
         <v>86</v>
@@ -4447,7 +4539,7 @@
         <v>104</v>
       </c>
       <c r="C21" s="42" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="D21" s="42" t="s">
         <v>89</v>
@@ -4479,7 +4571,7 @@
         <v>106</v>
       </c>
       <c r="C23" s="42" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="D23" s="42" t="s">
         <v>94</v>
@@ -4493,13 +4585,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="42" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C24" s="42" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="D24" s="42" t="s">
         <v>95</v>
@@ -4561,64 +4653,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="52.8" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="48" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="46"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="49"/>
+      <c r="I1" s="50"/>
     </row>
     <row r="2" spans="1:9" ht="28.8">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="45" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="45" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="45" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="48" t="s">
+      <c r="E2" s="45" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="48" t="s">
+      <c r="F2" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="48" t="s">
+      <c r="G2" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="48" t="s">
+      <c r="H2" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="I2" s="48" t="s">
+      <c r="I2" s="45" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="43.2">
-      <c r="A3" s="49" t="s">
-        <v>344</v>
-      </c>
-      <c r="B3" s="49" t="s">
-        <v>345</v>
-      </c>
-      <c r="C3" s="50">
+      <c r="A3" s="46" t="s">
+        <v>340</v>
+      </c>
+      <c r="B3" s="46" t="s">
+        <v>341</v>
+      </c>
+      <c r="C3" s="47">
         <v>8</v>
       </c>
-      <c r="D3" s="50">
+      <c r="D3" s="47">
         <v>8</v>
       </c>
-      <c r="E3" s="50">
+      <c r="E3" s="47">
         <v>0</v>
       </c>
-      <c r="F3" s="50">
+      <c r="F3" s="47">
         <v>8</v>
       </c>
       <c r="G3" s="3">
@@ -4632,20 +4724,20 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="43.2">
-      <c r="A4" s="49"/>
-      <c r="B4" s="49" t="s">
-        <v>346</v>
-      </c>
-      <c r="C4" s="50">
+      <c r="A4" s="46"/>
+      <c r="B4" s="46" t="s">
+        <v>342</v>
+      </c>
+      <c r="C4" s="47">
         <v>8</v>
       </c>
-      <c r="D4" s="50">
+      <c r="D4" s="47">
         <v>8</v>
       </c>
-      <c r="E4" s="50">
+      <c r="E4" s="47">
         <v>0</v>
       </c>
-      <c r="F4" s="50">
+      <c r="F4" s="47">
         <v>8</v>
       </c>
       <c r="G4" s="3">
@@ -4659,20 +4751,20 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="28.8">
-      <c r="A5" s="49"/>
-      <c r="B5" s="49" t="s">
-        <v>347</v>
-      </c>
-      <c r="C5" s="50">
+      <c r="A5" s="46"/>
+      <c r="B5" s="46" t="s">
+        <v>343</v>
+      </c>
+      <c r="C5" s="47">
         <v>6</v>
       </c>
-      <c r="D5" s="50">
+      <c r="D5" s="47">
         <v>6</v>
       </c>
-      <c r="E5" s="50">
+      <c r="E5" s="47">
         <v>0</v>
       </c>
-      <c r="F5" s="50">
+      <c r="F5" s="47">
         <v>6</v>
       </c>
       <c r="G5" s="3">
@@ -4686,20 +4778,20 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="28.8">
-      <c r="A6" s="49"/>
-      <c r="B6" s="49" t="s">
-        <v>348</v>
-      </c>
-      <c r="C6" s="50">
+      <c r="A6" s="46"/>
+      <c r="B6" s="46" t="s">
+        <v>344</v>
+      </c>
+      <c r="C6" s="47">
         <v>3</v>
       </c>
-      <c r="D6" s="50">
+      <c r="D6" s="47">
         <v>3</v>
       </c>
-      <c r="E6" s="50">
+      <c r="E6" s="47">
         <v>0</v>
       </c>
-      <c r="F6" s="50">
+      <c r="F6" s="47">
         <v>3</v>
       </c>
       <c r="G6" s="3">

</xml_diff>

<commit_message>
Added few new features
</commit_message>
<xml_diff>
--- a/Day 2_Manual Testing/Sayan_Saha_Magicbricks_Group4.xlsx
+++ b/Day 2_Manual Testing/Sayan_Saha_Magicbricks_Group4.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sayan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Sprint_Group_4_Magicbricks_edit\Day 2_Manual Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF04AD86-B9E4-44FE-BBDF-97351F52B79C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020DD4EC-4297-4F51-AA35-DA62C66CECA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="11496" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Story_Edited" sheetId="8" r:id="rId1"/>
@@ -836,9 +836,6 @@
     <t>Tab: Plot
 Plot Area Min: 2000 sq yards
 Plot Area Max: 500 sq yards (inverted)</t>
-  </si>
-  <si>
-    <t>Search not executed. Validation error: 'Minimum area cannot be greater than maximum area'. Fields highlighted in error state. No results loaded.</t>
   </si>
   <si>
     <t>Verify Commercial tab shows Rent/Lease sub-options with Office Space Type filter and returns only commercial listings</t>
@@ -1428,6 +1425,9 @@
   </si>
   <si>
     <t>Test Case Passed Successfully</t>
+  </si>
+  <si>
+    <t>Search not executed. As the Max Plot Area is less than the Min Plot Area , the Plot Area Max is changed to Maximum keeping the Plot Area Min intact.</t>
   </si>
 </sst>
 </file>
@@ -1874,17 +1874,17 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2216,7 +2216,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>4</v>
@@ -2227,7 +2227,7 @@
         <v>8</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C5" s="9" t="s">
         <v>4</v>
@@ -2238,7 +2238,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C6" s="9" t="s">
         <v>4</v>
@@ -2249,7 +2249,7 @@
         <v>110</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C7" s="9" t="s">
         <v>11</v>
@@ -2260,7 +2260,7 @@
         <v>111</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C8" s="9" t="s">
         <v>11</v>
@@ -2282,7 +2282,7 @@
         <v>113</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C10" s="9" t="s">
         <v>4</v>
@@ -2293,7 +2293,7 @@
         <v>114</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C11" s="9" t="s">
         <v>4</v>
@@ -2304,7 +2304,7 @@
         <v>115</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C12" s="9" t="s">
         <v>4</v>
@@ -2315,7 +2315,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C13" s="9" t="s">
         <v>4</v>
@@ -2326,7 +2326,7 @@
         <v>117</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>4</v>
@@ -2337,7 +2337,7 @@
         <v>118</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>4</v>
@@ -2411,10 +2411,10 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="33" t="s">
+        <v>302</v>
+      </c>
+      <c r="B22" s="34" t="s">
         <v>303</v>
-      </c>
-      <c r="B22" s="34" t="s">
-        <v>304</v>
       </c>
       <c r="C22" s="33" t="s">
         <v>4</v>
@@ -2422,10 +2422,10 @@
     </row>
     <row r="23" spans="1:3" ht="27.6">
       <c r="A23" s="35" t="s">
+        <v>304</v>
+      </c>
+      <c r="B23" s="36" t="s">
         <v>305</v>
-      </c>
-      <c r="B23" s="36" t="s">
-        <v>306</v>
       </c>
       <c r="C23" s="35" t="s">
         <v>4</v>
@@ -2433,10 +2433,10 @@
     </row>
     <row r="24" spans="1:3" ht="43.2">
       <c r="A24" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="B24" s="8" t="s">
         <v>307</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>308</v>
       </c>
       <c r="C24" s="38" t="s">
         <v>4</v>
@@ -2444,10 +2444,10 @@
     </row>
     <row r="25" spans="1:3" ht="43.2">
       <c r="A25" s="37" t="s">
+        <v>308</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>309</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>310</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>4</v>
@@ -2455,10 +2455,10 @@
     </row>
     <row r="26" spans="1:3" ht="43.2">
       <c r="A26" s="37" t="s">
+        <v>310</v>
+      </c>
+      <c r="B26" s="8" t="s">
         <v>311</v>
-      </c>
-      <c r="B26" s="8" t="s">
-        <v>312</v>
       </c>
       <c r="C26" s="38" t="s">
         <v>11</v>
@@ -2485,7 +2485,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="82.8" customHeight="1">
       <c r="A1" s="20" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B1" s="20" t="s">
         <v>12</v>
@@ -2497,7 +2497,7 @@
         <v>14</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F1" s="20" t="s">
         <v>15</v>
@@ -2505,7 +2505,7 @@
     </row>
     <row r="2" spans="1:6" ht="151.80000000000001" customHeight="1">
       <c r="A2" s="39" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B2" s="39" t="s">
         <v>50</v>
@@ -2514,18 +2514,18 @@
         <v>51</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E2" s="18">
         <v>1</v>
       </c>
       <c r="F2" s="19" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="256.2" customHeight="1">
       <c r="A3" s="39" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B3" s="39" t="s">
         <v>54</v>
@@ -2534,18 +2534,18 @@
         <v>55</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E3" s="18">
         <v>2</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="117" customHeight="1">
       <c r="A4" s="39" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B4" s="39" t="s">
         <v>58</v>
@@ -2554,18 +2554,18 @@
         <v>59</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E4" s="18">
         <v>2</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="54.6" customHeight="1">
       <c r="A5" s="39" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B5" s="39" t="s">
         <v>62</v>
@@ -2574,18 +2574,18 @@
         <v>63</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E5" s="18">
         <v>1</v>
       </c>
       <c r="F5" s="19" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="79.2" customHeight="1">
       <c r="A6" s="39" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B6" s="39" t="s">
         <v>66</v>
@@ -2594,18 +2594,18 @@
         <v>67</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E6" s="18">
         <v>2</v>
       </c>
       <c r="F6" s="19" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="87" customHeight="1">
       <c r="A7" s="39" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B7" s="39" t="s">
         <v>70</v>
@@ -2614,18 +2614,18 @@
         <v>71</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E7" s="18">
         <v>1</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="67.8" customHeight="1">
       <c r="A8" s="39" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B8" s="39" t="s">
         <v>74</v>
@@ -2634,18 +2634,18 @@
         <v>75</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E8" s="18">
         <v>1</v>
       </c>
       <c r="F8" s="19" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="84" customHeight="1">
       <c r="A9" s="39" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B9" s="39" t="s">
         <v>78</v>
@@ -2654,18 +2654,18 @@
         <v>79</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E9" s="18">
         <v>1</v>
       </c>
       <c r="F9" s="19" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="82.2" customHeight="1">
       <c r="A10" s="39" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B10" s="39" t="s">
         <v>83</v>
@@ -2674,18 +2674,18 @@
         <v>84</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E10" s="18">
         <v>2</v>
       </c>
       <c r="F10" s="19" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="85.2" customHeight="1">
       <c r="A11" s="39" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B11" s="39" t="s">
         <v>87</v>
@@ -2694,18 +2694,18 @@
         <v>88</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E11" s="18">
         <v>2</v>
       </c>
       <c r="F11" s="19" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="88.2" customHeight="1">
       <c r="A12" s="39" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B12" s="39" t="s">
         <v>92</v>
@@ -2714,18 +2714,18 @@
         <v>93</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E12" s="18">
         <v>1</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="99.6" customHeight="1">
       <c r="A13" s="39" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B13" s="39" t="s">
         <v>96</v>
@@ -2734,18 +2734,18 @@
         <v>97</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E13" s="18">
         <v>1</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="94.2" customHeight="1">
       <c r="A14" s="39" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B14" s="39" t="s">
         <v>100</v>
@@ -2754,18 +2754,18 @@
         <v>101</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E14" s="18">
         <v>1</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="61.8" customHeight="1">
       <c r="A15" s="39" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B15" s="39" t="s">
         <v>102</v>
@@ -2774,18 +2774,18 @@
         <v>103</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E15" s="18">
         <v>1</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="95.4" hidden="1" customHeight="1">
       <c r="A16" s="39" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B16" s="39" t="s">
         <v>104</v>
@@ -2794,18 +2794,18 @@
         <v>105</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E16" s="18">
         <v>2</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="91.8" customHeight="1">
       <c r="A17" s="39" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B17" s="39" t="s">
         <v>106</v>
@@ -2814,33 +2814,33 @@
         <v>107</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E17" s="18">
         <v>1</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="72" customHeight="1">
       <c r="A18" s="39" t="s">
+        <v>312</v>
+      </c>
+      <c r="B18" s="39" t="s">
         <v>313</v>
       </c>
-      <c r="B18" s="39" t="s">
-        <v>314</v>
-      </c>
       <c r="C18" s="19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E18" s="18">
         <v>3</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="94.8" customHeight="1"/>
@@ -2937,7 +2937,7 @@
     </row>
     <row r="2" spans="1:13" ht="72">
       <c r="A2" s="22" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B2" s="23"/>
       <c r="C2" s="23"/>
@@ -2974,14 +2974,14 @@
       <c r="G3" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="H3" s="51" t="s">
-        <v>351</v>
+      <c r="H3" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I3" s="24"/>
       <c r="J3" s="25"/>
       <c r="K3" s="24"/>
       <c r="L3" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M3" s="24" t="s">
         <v>50</v>
@@ -2989,7 +2989,7 @@
     </row>
     <row r="4" spans="1:13" ht="72">
       <c r="A4" s="22" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
@@ -3026,14 +3026,14 @@
       <c r="G5" s="27" t="s">
         <v>145</v>
       </c>
-      <c r="H5" s="51" t="s">
-        <v>351</v>
+      <c r="H5" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I5" s="28"/>
       <c r="J5" s="27"/>
       <c r="K5" s="28"/>
       <c r="L5" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M5" s="28" t="s">
         <v>54</v>
@@ -3061,14 +3061,14 @@
       <c r="G6" s="30" t="s">
         <v>149</v>
       </c>
-      <c r="H6" s="52" t="s">
-        <v>351</v>
+      <c r="H6" s="49" t="s">
+        <v>350</v>
       </c>
       <c r="I6" s="29"/>
       <c r="J6" s="30"/>
       <c r="K6" s="29"/>
       <c r="L6" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M6" s="29" t="s">
         <v>54</v>
@@ -3076,7 +3076,7 @@
     </row>
     <row r="7" spans="1:13" ht="72">
       <c r="A7" s="22" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="26"/>
@@ -3113,14 +3113,14 @@
       <c r="G8" s="27" t="s">
         <v>155</v>
       </c>
-      <c r="H8" s="51" t="s">
-        <v>351</v>
+      <c r="H8" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I8" s="28"/>
       <c r="J8" s="27"/>
       <c r="K8" s="28"/>
       <c r="L8" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M8" s="28" t="s">
         <v>58</v>
@@ -3148,14 +3148,14 @@
       <c r="G9" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="H9" s="52" t="s">
-        <v>351</v>
+      <c r="H9" s="49" t="s">
+        <v>350</v>
       </c>
       <c r="I9" s="29"/>
       <c r="J9" s="30"/>
       <c r="K9" s="29"/>
       <c r="L9" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M9" s="29" t="s">
         <v>58</v>
@@ -3163,7 +3163,7 @@
     </row>
     <row r="10" spans="1:13" ht="84">
       <c r="A10" s="22" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B10" s="26"/>
       <c r="C10" s="26"/>
@@ -3200,14 +3200,14 @@
       <c r="G11" s="27" t="s">
         <v>165</v>
       </c>
-      <c r="H11" s="51" t="s">
-        <v>351</v>
+      <c r="H11" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I11" s="28"/>
       <c r="J11" s="27"/>
       <c r="K11" s="28"/>
       <c r="L11" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M11" s="28" t="s">
         <v>62</v>
@@ -3215,7 +3215,7 @@
     </row>
     <row r="12" spans="1:13" ht="84">
       <c r="A12" s="22" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B12" s="26"/>
       <c r="C12" s="26"/>
@@ -3244,22 +3244,22 @@
         <v>168</v>
       </c>
       <c r="E13" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="F13" s="25" t="s">
         <v>352</v>
-      </c>
-      <c r="F13" s="25" t="s">
-        <v>353</v>
       </c>
       <c r="G13" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="H13" s="51" t="s">
-        <v>351</v>
+      <c r="H13" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I13" s="24"/>
       <c r="J13" s="25"/>
       <c r="K13" s="24"/>
       <c r="L13" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M13" s="24" t="s">
         <v>66</v>
@@ -3287,14 +3287,14 @@
       <c r="G14" s="31" t="s">
         <v>173</v>
       </c>
-      <c r="H14" s="52" t="s">
-        <v>351</v>
+      <c r="H14" s="49" t="s">
+        <v>350</v>
       </c>
       <c r="I14" s="32"/>
       <c r="J14" s="31"/>
       <c r="K14" s="32"/>
       <c r="L14" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M14" s="32" t="s">
         <v>66</v>
@@ -3302,7 +3302,7 @@
     </row>
     <row r="15" spans="1:13" ht="84">
       <c r="A15" s="22" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -3339,14 +3339,14 @@
       <c r="G16" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="H16" s="51" t="s">
-        <v>351</v>
+      <c r="H16" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I16" s="24"/>
       <c r="J16" s="25"/>
       <c r="K16" s="24"/>
       <c r="L16" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M16" s="24" t="s">
         <v>70</v>
@@ -3354,7 +3354,7 @@
     </row>
     <row r="17" spans="1:13" ht="84">
       <c r="A17" s="22" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
@@ -3391,14 +3391,14 @@
       <c r="G18" s="25" t="s">
         <v>185</v>
       </c>
-      <c r="H18" s="51" t="s">
-        <v>351</v>
+      <c r="H18" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I18" s="24"/>
       <c r="J18" s="25"/>
       <c r="K18" s="24"/>
       <c r="L18" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M18" s="24" t="s">
         <v>74</v>
@@ -3406,7 +3406,7 @@
     </row>
     <row r="19" spans="1:13" ht="60">
       <c r="A19" s="22" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -3443,14 +3443,14 @@
       <c r="G20" s="27" t="s">
         <v>190</v>
       </c>
-      <c r="H20" s="51" t="s">
-        <v>351</v>
+      <c r="H20" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I20" s="28"/>
       <c r="J20" s="27"/>
       <c r="K20" s="28"/>
       <c r="L20" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M20" s="28" t="s">
         <v>78</v>
@@ -3458,7 +3458,7 @@
     </row>
     <row r="21" spans="1:13" ht="84">
       <c r="A21" s="22" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B21" s="26"/>
       <c r="C21" s="26"/>
@@ -3495,14 +3495,14 @@
       <c r="G22" s="25" t="s">
         <v>196</v>
       </c>
-      <c r="H22" s="51" t="s">
-        <v>351</v>
+      <c r="H22" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I22" s="24"/>
       <c r="J22" s="25"/>
       <c r="K22" s="24"/>
       <c r="L22" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M22" s="24" t="s">
         <v>83</v>
@@ -3525,19 +3525,19 @@
         <v>198</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G23" s="31" t="s">
         <v>199</v>
       </c>
-      <c r="H23" s="52" t="s">
-        <v>351</v>
+      <c r="H23" s="49" t="s">
+        <v>350</v>
       </c>
       <c r="I23" s="32"/>
       <c r="J23" s="31"/>
       <c r="K23" s="32"/>
       <c r="L23" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M23" s="32" t="s">
         <v>83</v>
@@ -3545,7 +3545,7 @@
     </row>
     <row r="24" spans="1:13" ht="84">
       <c r="A24" s="22" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B24" s="26"/>
       <c r="C24" s="26"/>
@@ -3574,22 +3574,22 @@
         <v>202</v>
       </c>
       <c r="E25" s="25" t="s">
+        <v>353</v>
+      </c>
+      <c r="F25" s="25" t="s">
         <v>354</v>
-      </c>
-      <c r="F25" s="25" t="s">
-        <v>355</v>
       </c>
       <c r="G25" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="H25" s="51" t="s">
-        <v>351</v>
+      <c r="H25" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I25" s="24"/>
       <c r="J25" s="25"/>
       <c r="K25" s="24"/>
       <c r="L25" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M25" s="24" t="s">
         <v>87</v>
@@ -3617,14 +3617,14 @@
       <c r="G26" s="31" t="s">
         <v>206</v>
       </c>
-      <c r="H26" s="52" t="s">
-        <v>351</v>
+      <c r="H26" s="49" t="s">
+        <v>350</v>
       </c>
       <c r="I26" s="32"/>
       <c r="J26" s="31"/>
       <c r="K26" s="32"/>
       <c r="L26" s="29" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M26" s="32" t="s">
         <v>87</v>
@@ -3632,7 +3632,7 @@
     </row>
     <row r="27" spans="1:13" ht="84">
       <c r="A27" s="22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -3669,14 +3669,14 @@
       <c r="G28" s="25" t="s">
         <v>212</v>
       </c>
-      <c r="H28" s="51" t="s">
-        <v>351</v>
+      <c r="H28" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I28" s="24"/>
       <c r="J28" s="25"/>
       <c r="K28" s="24"/>
       <c r="L28" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M28" s="24" t="s">
         <v>92</v>
@@ -3684,7 +3684,7 @@
     </row>
     <row r="29" spans="1:13" ht="72">
       <c r="A29" s="22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B29" s="23"/>
       <c r="C29" s="23"/>
@@ -3721,14 +3721,14 @@
       <c r="G30" s="25" t="s">
         <v>218</v>
       </c>
-      <c r="H30" s="51" t="s">
-        <v>351</v>
+      <c r="H30" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I30" s="24"/>
       <c r="J30" s="25"/>
       <c r="K30" s="24"/>
       <c r="L30" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M30" s="24" t="s">
         <v>96</v>
@@ -3736,7 +3736,7 @@
     </row>
     <row r="31" spans="1:13" ht="72">
       <c r="A31" s="22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B31" s="26"/>
       <c r="C31" s="26"/>
@@ -3773,14 +3773,14 @@
       <c r="G32" s="27" t="s">
         <v>223</v>
       </c>
-      <c r="H32" s="51" t="s">
-        <v>351</v>
+      <c r="H32" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I32" s="28"/>
       <c r="J32" s="27"/>
       <c r="K32" s="28"/>
       <c r="L32" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M32" s="28" t="s">
         <v>100</v>
@@ -3788,7 +3788,7 @@
     </row>
     <row r="33" spans="1:13" ht="84">
       <c r="A33" s="22" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B33" s="26"/>
       <c r="C33" s="26"/>
@@ -3825,14 +3825,14 @@
       <c r="G34" s="25" t="s">
         <v>229</v>
       </c>
-      <c r="H34" s="51" t="s">
-        <v>351</v>
+      <c r="H34" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I34" s="24"/>
       <c r="J34" s="25"/>
       <c r="K34" s="24"/>
       <c r="L34" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M34" s="24" t="s">
         <v>102</v>
@@ -3840,7 +3840,7 @@
     </row>
     <row r="35" spans="1:13" ht="72">
       <c r="A35" s="22" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B35" s="23"/>
       <c r="C35" s="23"/>
@@ -3877,14 +3877,14 @@
       <c r="G36" s="25" t="s">
         <v>234</v>
       </c>
-      <c r="H36" s="51" t="s">
-        <v>351</v>
+      <c r="H36" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I36" s="24"/>
       <c r="J36" s="25"/>
       <c r="K36" s="24"/>
       <c r="L36" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M36" s="24" t="s">
         <v>104</v>
@@ -3910,16 +3910,16 @@
         <v>237</v>
       </c>
       <c r="G37" s="25" t="s">
-        <v>238</v>
-      </c>
-      <c r="H37" s="51" t="s">
-        <v>351</v>
+        <v>356</v>
+      </c>
+      <c r="H37" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I37" s="24"/>
       <c r="J37" s="25"/>
       <c r="K37" s="24"/>
       <c r="L37" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M37" s="24" t="s">
         <v>104</v>
@@ -3927,7 +3927,7 @@
     </row>
     <row r="38" spans="1:13" ht="84">
       <c r="A38" s="22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B38" s="23"/>
       <c r="C38" s="23"/>
@@ -3947,31 +3947,31 @@
         <v>94</v>
       </c>
       <c r="B39" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="C39" s="25" t="s">
         <v>239</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="D39" s="25" t="s">
         <v>240</v>
       </c>
-      <c r="D39" s="25" t="s">
+      <c r="E39" s="25" t="s">
         <v>241</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="F39" s="25" t="s">
         <v>242</v>
       </c>
-      <c r="F39" s="25" t="s">
+      <c r="G39" s="25" t="s">
         <v>243</v>
       </c>
-      <c r="G39" s="25" t="s">
-        <v>244</v>
-      </c>
-      <c r="H39" s="51" t="s">
-        <v>351</v>
+      <c r="H39" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I39" s="24"/>
       <c r="J39" s="25"/>
       <c r="K39" s="24"/>
       <c r="L39" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M39" s="24" t="s">
         <v>106</v>
@@ -3979,7 +3979,7 @@
     </row>
     <row r="40" spans="1:13" ht="60">
       <c r="A40" s="40" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B40" s="23"/>
       <c r="C40" s="23"/>
@@ -3999,34 +3999,34 @@
         <v>95</v>
       </c>
       <c r="B41" s="27" t="s">
+        <v>320</v>
+      </c>
+      <c r="C41" s="27" t="s">
         <v>321</v>
       </c>
-      <c r="C41" s="27" t="s">
+      <c r="D41" s="27" t="s">
         <v>322</v>
       </c>
-      <c r="D41" s="27" t="s">
+      <c r="E41" s="27" t="s">
         <v>323</v>
       </c>
-      <c r="E41" s="27" t="s">
+      <c r="F41" s="27" t="s">
         <v>324</v>
       </c>
-      <c r="F41" s="27" t="s">
+      <c r="G41" s="27" t="s">
         <v>325</v>
       </c>
-      <c r="G41" s="27" t="s">
-        <v>326</v>
-      </c>
-      <c r="H41" s="51" t="s">
-        <v>351</v>
+      <c r="H41" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I41" s="27"/>
       <c r="J41" s="27"/>
       <c r="K41" s="27"/>
       <c r="L41" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M41" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="198">
@@ -4034,34 +4034,34 @@
         <v>98</v>
       </c>
       <c r="B42" s="27" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C42" s="27" t="s">
+        <v>326</v>
+      </c>
+      <c r="D42" s="27" t="s">
         <v>327</v>
       </c>
-      <c r="D42" s="27" t="s">
+      <c r="E42" s="27" t="s">
         <v>328</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="F42" s="27" t="s">
         <v>329</v>
       </c>
-      <c r="F42" s="27" t="s">
+      <c r="G42" s="27" t="s">
         <v>330</v>
       </c>
-      <c r="G42" s="27" t="s">
-        <v>331</v>
-      </c>
-      <c r="H42" s="51" t="s">
-        <v>351</v>
+      <c r="H42" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I42" s="27"/>
       <c r="J42" s="27"/>
       <c r="K42" s="27"/>
       <c r="L42" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M42" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="184.8">
@@ -4069,34 +4069,34 @@
         <v>99</v>
       </c>
       <c r="B43" s="27" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="D43" s="27" t="s">
+        <v>331</v>
+      </c>
+      <c r="E43" s="27" t="s">
         <v>332</v>
       </c>
-      <c r="E43" s="27" t="s">
+      <c r="F43" s="27" t="s">
         <v>333</v>
       </c>
-      <c r="F43" s="27" t="s">
+      <c r="G43" s="27" t="s">
         <v>334</v>
       </c>
-      <c r="G43" s="27" t="s">
-        <v>335</v>
-      </c>
-      <c r="H43" s="51" t="s">
-        <v>351</v>
+      <c r="H43" s="48" t="s">
+        <v>350</v>
       </c>
       <c r="I43" s="27"/>
       <c r="J43" s="27"/>
       <c r="K43" s="27"/>
       <c r="L43" s="24" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M43" s="28" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>
@@ -4140,22 +4140,22 @@
     </row>
     <row r="2" spans="1:6" ht="69.900000000000006" customHeight="1">
       <c r="A2" s="42" t="s">
+        <v>335</v>
+      </c>
+      <c r="B2" s="42" t="s">
         <v>336</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="C2" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="42" t="s">
+        <v>335</v>
+      </c>
+      <c r="E2" s="43" t="s">
+        <v>335</v>
+      </c>
+      <c r="F2" s="42" t="s">
         <v>338</v>
-      </c>
-      <c r="D2" s="42" t="s">
-        <v>336</v>
-      </c>
-      <c r="E2" s="43" t="s">
-        <v>336</v>
-      </c>
-      <c r="F2" s="42" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -4207,13 +4207,13 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="42" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B2" s="42" t="s">
         <v>50</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D2" s="42" t="s">
         <v>49</v>
@@ -4231,7 +4231,7 @@
         <v>54</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D3" s="42" t="s">
         <v>52</v>
@@ -4263,7 +4263,7 @@
         <v>58</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D5" s="42" t="s">
         <v>56</v>
@@ -4295,7 +4295,7 @@
         <v>62</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D7" s="42" t="s">
         <v>60</v>
@@ -4313,7 +4313,7 @@
         <v>66</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D8" s="42" t="s">
         <v>61</v>
@@ -4341,13 +4341,13 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="42" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="B10" s="42" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D10" s="42" t="s">
         <v>65</v>
@@ -4365,7 +4365,7 @@
         <v>74</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D11" s="42" t="s">
         <v>68</v>
@@ -4383,7 +4383,7 @@
         <v>78</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D12" s="42" t="s">
         <v>69</v>
@@ -4401,7 +4401,7 @@
         <v>83</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D13" s="42" t="s">
         <v>72</v>
@@ -4433,7 +4433,7 @@
         <v>87</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D15" s="42" t="s">
         <v>76</v>
@@ -4465,7 +4465,7 @@
         <v>92</v>
       </c>
       <c r="C17" s="42" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D17" s="42" t="s">
         <v>81</v>
@@ -4479,13 +4479,13 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="42" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="B18" s="42" t="s">
         <v>96</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D18" s="42" t="s">
         <v>82</v>
@@ -4503,7 +4503,7 @@
         <v>100</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D19" s="42" t="s">
         <v>85</v>
@@ -4521,7 +4521,7 @@
         <v>102</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D20" s="42" t="s">
         <v>86</v>
@@ -4539,7 +4539,7 @@
         <v>104</v>
       </c>
       <c r="C21" s="42" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D21" s="42" t="s">
         <v>89</v>
@@ -4571,7 +4571,7 @@
         <v>106</v>
       </c>
       <c r="C23" s="42" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D23" s="42" t="s">
         <v>94</v>
@@ -4585,13 +4585,13 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="42" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C24" s="42" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="D24" s="42" t="s">
         <v>95</v>
@@ -4653,17 +4653,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="52.8" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="50" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="50"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="52"/>
     </row>
     <row r="2" spans="1:9" ht="28.8">
       <c r="A2" s="44" t="s">
@@ -4696,10 +4696,10 @@
     </row>
     <row r="3" spans="1:9" ht="43.2">
       <c r="A3" s="46" t="s">
+        <v>339</v>
+      </c>
+      <c r="B3" s="46" t="s">
         <v>340</v>
-      </c>
-      <c r="B3" s="46" t="s">
-        <v>341</v>
       </c>
       <c r="C3" s="47">
         <v>8</v>
@@ -4726,7 +4726,7 @@
     <row r="4" spans="1:9" ht="43.2">
       <c r="A4" s="46"/>
       <c r="B4" s="46" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C4" s="47">
         <v>8</v>
@@ -4753,7 +4753,7 @@
     <row r="5" spans="1:9" ht="28.8">
       <c r="A5" s="46"/>
       <c r="B5" s="46" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C5" s="47">
         <v>6</v>
@@ -4780,7 +4780,7 @@
     <row r="6" spans="1:9" ht="28.8">
       <c r="A6" s="46"/>
       <c r="B6" s="46" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C6" s="47">
         <v>3</v>

</xml_diff>